<commit_message>
Fix TEV pack: use official TO number, default Appendix 47 checkbox, add ATR letterhead and admin approver reassignment
</commit_message>
<xml_diff>
--- a/resources/templates/TEV_TEMPLATE.xlsx
+++ b/resources/templates/TEV_TEMPLATE.xlsx
@@ -877,6 +877,41 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6762750" cy="1257300"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="image1.png" descr="A close-up of a white background&#10;&#10;AI-generated content may be incorrect."/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="0"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>

</xml_diff>